<commit_message>
Scenario 2 Write a LINQ query to update the "Price" column value by 50
</commit_message>
<xml_diff>
--- a/uipath_linq_filter_example.xlsx
+++ b/uipath_linq_filter_example.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\revision\UiPath Practice\LinqExcelOperation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEC73172-3720-4A63-82C6-C17F8072DA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783A4A58-1B95-4CE3-A728-B9DD6BC4B531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="InputData" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="SumSheet" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t>Total</t>
   </si>
@@ -115,6 +117,24 @@
   </si>
   <si>
     <t>1200 INR</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Grapes</t>
   </si>
 </sst>
 </file>
@@ -158,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -171,6 +191,12 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -606,4 +632,112 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9194E911-48BB-4152-BC29-D2E7496EEDAC}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="6">
+        <v>3</v>
+      </c>
+      <c r="C2" s="6">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="6">
+        <v>2</v>
+      </c>
+      <c r="C3" s="6">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="6">
+        <v>1</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFF6D7AA-C8F0-405F-821A-83238D51E7D5}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="C2">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Use of DotFirst Method
</commit_message>
<xml_diff>
--- a/uipath_linq_filter_example.xlsx
+++ b/uipath_linq_filter_example.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\revision\UiPath Practice\LinqExcelOperation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F07E391-13A5-426E-9BB8-0189D50AA991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E86DF2-C607-4009-A9D8-37CFEC29449B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="4800" yWindow="2810" windowWidth="14400" windowHeight="7270" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="InputData" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
     <sheet name="SumSheet" sheetId="3" r:id="rId3"/>
     <sheet name="sumspecific" sheetId="4" r:id="rId4"/>
+    <sheet name="RemoveExtraSpace" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="63">
   <si>
     <t>Total</t>
   </si>
@@ -136,6 +137,93 @@
   </si>
   <si>
     <t>Grapes</t>
+  </si>
+  <si>
+    <t>Invoice Number</t>
+  </si>
+  <si>
+    <t>Vendor Tax ID</t>
+  </si>
+  <si>
+    <t>FR453231</t>
+  </si>
+  <si>
+    <t>Waste management se</t>
+  </si>
+  <si>
+    <t>163433 EUR</t>
+  </si>
+  <si>
+    <t>Beverages and Caterin</t>
+  </si>
+  <si>
+    <t>174892 RON</t>
+  </si>
+  <si>
+    <t>IT231232</t>
+  </si>
+  <si>
+    <t>Concierge Services</t>
+  </si>
+  <si>
+    <t>124835 CAD</t>
+  </si>
+  <si>
+    <t>RO123456</t>
+  </si>
+  <si>
+    <t>120845 USD</t>
+  </si>
+  <si>
+    <t>FR329083</t>
+  </si>
+  <si>
+    <t>Professional Services</t>
+  </si>
+  <si>
+    <t>195704 RON</t>
+  </si>
+  <si>
+    <t>DE763212</t>
+  </si>
+  <si>
+    <t>81872.4 EUR</t>
+  </si>
+  <si>
+    <t>RU567434</t>
+  </si>
+  <si>
+    <t>38084.4 EUR</t>
+  </si>
+  <si>
+    <t>RO125678</t>
+  </si>
+  <si>
+    <t>242988 EUR</t>
+  </si>
+  <si>
+    <t>0000-00-00</t>
+  </si>
+  <si>
+    <t>259774 EUR</t>
+  </si>
+  <si>
+    <t>RO892123</t>
+  </si>
+  <si>
+    <t>15524.4 USD</t>
+  </si>
+  <si>
+    <t>RO874232</t>
+  </si>
+  <si>
+    <t>333860 CAD</t>
+  </si>
+  <si>
+    <t>FR065748</t>
+  </si>
+  <si>
+    <t>1830 RON</t>
   </si>
 </sst>
 </file>
@@ -179,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -199,6 +287,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -691,7 +780,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFF6D7AA-C8F0-405F-821A-83238D51E7D5}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -779,6 +868,94 @@
         <v>1</v>
       </c>
       <c r="C8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
         <v>100</v>
       </c>
     </row>
@@ -789,7 +966,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D841F88-5A01-452B-B03B-DCF3D9ECD539}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -836,6 +1013,552 @@
         <v>50</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{970E0ED4-45C9-4ABC-8E1B-B4C2686CEA0A}">
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="5" width="27.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>334450</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="7">
+        <v>41666</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>381388</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="7">
+        <v>41649</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>505578</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="7">
+        <v>41659</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>515397</v>
+      </c>
+      <c r="B5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="7">
+        <v>41663</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>675814</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="7">
+        <v>41660</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>266679</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="7">
+        <v>41642</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>356850</v>
+      </c>
+      <c r="B8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="7">
+        <v>41645</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>380288</v>
+      </c>
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>758324</v>
+      </c>
+      <c r="B10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="7">
+        <v>41646</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>520639</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="7">
+        <v>41660</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>990481</v>
+      </c>
+      <c r="B12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="7">
+        <v>41662</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>861123</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="7">
+        <v>41662</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>334450</v>
+      </c>
+      <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15">
+        <v>163433</v>
+      </c>
+      <c r="E15" s="7">
+        <v>41666</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>381388</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16">
+        <v>174892</v>
+      </c>
+      <c r="E16" s="7">
+        <v>41649</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>505578</v>
+      </c>
+      <c r="B17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17">
+        <v>124835</v>
+      </c>
+      <c r="E17" s="7">
+        <v>41659</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>515397</v>
+      </c>
+      <c r="B18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18">
+        <v>120845</v>
+      </c>
+      <c r="E18" s="7">
+        <v>41663</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>675814</v>
+      </c>
+      <c r="B19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19">
+        <v>195704</v>
+      </c>
+      <c r="E19" s="7">
+        <v>41660</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>266679</v>
+      </c>
+      <c r="B20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20">
+        <v>81872.399999999994</v>
+      </c>
+      <c r="E20" s="7">
+        <v>41642</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>356850</v>
+      </c>
+      <c r="B21" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21">
+        <v>38084.400000000001</v>
+      </c>
+      <c r="E21" s="7">
+        <v>41645</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>380288</v>
+      </c>
+      <c r="B22" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22">
+        <v>242988</v>
+      </c>
+      <c r="E22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>758324</v>
+      </c>
+      <c r="B23" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23">
+        <v>259774</v>
+      </c>
+      <c r="E23" s="7">
+        <v>41646</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>520639</v>
+      </c>
+      <c r="B24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24">
+        <v>15524.4</v>
+      </c>
+      <c r="E24" s="7">
+        <v>41660</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>990481</v>
+      </c>
+      <c r="B25" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25">
+        <v>333860</v>
+      </c>
+      <c r="E25" s="7">
+        <v>41662</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>861123</v>
+      </c>
+      <c r="B26" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" t="s">
+        <v>42</v>
+      </c>
+      <c r="D26">
+        <v>1830</v>
+      </c>
+      <c r="E26" s="7">
+        <v>41662</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated the code for filter the orange first occurance
</commit_message>
<xml_diff>
--- a/uipath_linq_filter_example.xlsx
+++ b/uipath_linq_filter_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\revision\UiPath Practice\LinqExcelOperation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E86DF2-C607-4009-A9D8-37CFEC29449B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E449314F-9C64-4169-86D3-B8974814DF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4800" yWindow="2810" windowWidth="14400" windowHeight="7270" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="InputData" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="SumSheet" sheetId="3" r:id="rId3"/>
     <sheet name="sumspecific" sheetId="4" r:id="rId4"/>
     <sheet name="RemoveExtraSpace" sheetId="5" r:id="rId5"/>
+    <sheet name="DotFirstMethod" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="69">
   <si>
     <t>Total</t>
   </si>
@@ -224,6 +225,24 @@
   </si>
   <si>
     <t>1830 RON</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>apple</t>
+  </si>
+  <si>
+    <t>orange</t>
+  </si>
+  <si>
+    <t>mango</t>
+  </si>
+  <si>
+    <t>kiwi</t>
+  </si>
+  <si>
+    <t>pear</t>
   </si>
 </sst>
 </file>
@@ -1562,4 +1581,80 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{446DC6C1-8D11-429B-90B8-55512F0BAD45}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>